<commit_message>
Sprint 6: Dashboard v2 - estrategia escalonada, portal cliente, upload documentos, coberturas pendientes
</commit_message>
<xml_diff>
--- a/DOCUMENTOS GENERALES/Inversion.xlsx
+++ b/DOCUMENTOS GENERALES/Inversion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1bed344dc1b8fd7e/Documentos/HedgePointMx/DOCUMENTOS GENERALES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{78B5CB14-704D-49DF-BE01-E037B069068D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6324E7CD-FAF5-4813-B504-E1EA6D37D50A}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{78B5CB14-704D-49DF-BE01-E037B069068D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59E87D41-ABAD-4CB2-970D-21DB3D7426D9}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2115" yWindow="810" windowWidth="10710" windowHeight="11970" xr2:uid="{87940882-4BE4-4A5D-B322-2E62A0CD040E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{87940882-4BE4-4A5D-B322-2E62A0CD040E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
   <si>
     <t>Claude PRO</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Chip Telcel</t>
   </si>
   <si>
-    <t>Celular</t>
-  </si>
-  <si>
     <t>DOMINIO 1 año</t>
   </si>
   <si>
@@ -80,9 +77,6 @@
     <t>Por hacer</t>
   </si>
   <si>
-    <t>Abogado</t>
-  </si>
-  <si>
     <t>Evento Emprendedores</t>
   </si>
   <si>
@@ -99,6 +93,12 @@
   </si>
   <si>
     <t>Bitwarden</t>
+  </si>
+  <si>
+    <t>Cita inicial con Abogados</t>
+  </si>
+  <si>
+    <t>Total=</t>
   </si>
 </sst>
 </file>
@@ -487,32 +487,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C3E4880-04E7-4677-92C4-FE3CA3A1ECE6}">
-  <dimension ref="A3:D21"/>
+  <dimension ref="A2:L20"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="19.53125" customWidth="1"/>
     <col min="3" max="3" width="12.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="K2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2">
+        <f>SUM(C5:C25)</f>
+        <v>11227</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>0</v>
@@ -524,9 +533,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>1</v>
@@ -538,12 +547,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1">
         <v>769</v>
@@ -552,9 +561,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>2</v>
@@ -566,9 +575,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>6</v>
@@ -580,91 +589,95 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C10" s="1">
+        <v>129</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3000</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C12" s="1">
+        <v>1749</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="1">
-        <v>1749</v>
+        <v>4000</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C14" s="1">
-        <v>4000</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A17" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" t="s">
-        <v>19</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
     </row>
@@ -686,12 +699,6 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>